<commit_message>
Add Good Saves by Quarter table + current-quarter callout, fix roadmap year wrap
Good Saves split into quarterly counts (Location/Q1-Q4/Annual table) and
current-quarter detail callout. Roadmap Q4→Q1 now increments the year.
Parser returns goodSavesByQuarter for both v1 (empty) and v2 layouts.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/qbu-intake-template-v2.xlsx
+++ b/public/qbu-intake-template-v2.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="136">
   <si>
     <t>COVER SLIDE</t>
   </si>
@@ -99,10 +99,13 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>GOOD SAVES</t>
-  </si>
-  <si>
-    <t>Hazards identified and prevented — these are reactive catches, not scheduled inspections.</t>
+    <t>GOOD SAVES BY QUARTER</t>
+  </si>
+  <si>
+    <t>GOOD SAVE DETAILS — CURRENT QUARTER</t>
+  </si>
+  <si>
+    <t>Hazards identified and prevented THIS QUARTER — reactive catches, not scheduled inspections.</t>
   </si>
   <si>
     <t>Hazard Prevented</t>
@@ -1084,7 +1087,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -1311,35 +1314,33 @@
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
     </row>
-    <row r="23" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-    </row>
-    <row r="24" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
+    <row r="23" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>31</v>
-      </c>
+      <c r="B23" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="7"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
@@ -1357,69 +1358,69 @@
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="7"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-    </row>
-    <row r="29" ht="8" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-    </row>
-    <row r="30" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-    </row>
-    <row r="31" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-    </row>
-    <row r="32" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
+    <row r="27" ht="8" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+    </row>
+    <row r="28" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="10"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+    </row>
+    <row r="30" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B32" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F32" s="6" t="s">
+      <c r="B30" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D30" s="6" t="s">
         <v>31</v>
       </c>
+      <c r="E30" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="7"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="7"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="7"/>
@@ -1437,13 +1438,77 @@
       <c r="E34" s="7"/>
       <c r="F34" s="7"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
+    <row r="35" ht="8" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="11"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+    </row>
+    <row r="38" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="7"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="7"/>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="7"/>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1462,7 +1527,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1472,7 +1537,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1505,7 +1570,7 @@
         <v>22</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1560,7 +1625,7 @@
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1570,7 +1635,7 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -1583,19 +1648,19 @@
         <v>18</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1650,7 +1715,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1660,7 +1725,7 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -1686,7 +1751,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1696,7 +1761,7 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -1770,7 +1835,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1779,7 +1844,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1795,87 +1860,87 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" ht="8" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -1887,7 +1952,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -1896,7 +1961,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -1912,7 +1977,7 @@
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1921,7 +1986,7 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -1930,121 +1995,121 @@
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -2064,43 +2129,43 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B2" s="8"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B3" s="16"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B4" s="16"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B5" s="16"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B6" s="16"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B7" s="16"/>
     </row>
@@ -2110,31 +2175,31 @@
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" s="11"/>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B10" s="8"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B11" s="16"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B12" s="16"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B13" s="16"/>
     </row>
@@ -2144,43 +2209,43 @@
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B15" s="10"/>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B16" s="8"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B17" s="16"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B18" s="16"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B19" s="16"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B20" s="16"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B21" s="16"/>
     </row>
@@ -2202,7 +2267,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2210,7 +2275,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2224,142 +2289,142 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" ht="8" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2370,7 +2435,7 @@
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -2378,7 +2443,7 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -2386,16 +2451,16 @@
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>18</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -2448,7 +2513,7 @@
     </row>
     <row r="26" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -2456,7 +2521,7 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -2467,13 +2532,13 @@
         <v>18</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -2517,14 +2582,14 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2539,10 +2604,10 @@
         <v>18</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2582,27 +2647,27 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -2642,7 +2707,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B1" s="1"/>
     </row>
@@ -2652,13 +2717,13 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B3" s="4"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B4" s="4"/>
     </row>
@@ -2668,48 +2733,48 @@
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B6" s="1"/>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" ht="8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -2718,37 +2783,37 @@
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B13" s="1"/>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B14" s="8"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B15" s="16"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B16" s="16"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B17" s="16"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B18" s="16"/>
     </row>
@@ -2768,14 +2833,14 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2787,13 +2852,13 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2833,60 +2898,60 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -2901,14 +2966,14 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>

</xml_diff>

<commit_message>
QBU deck review fixes — table titles, audit labels, pie chart per-location, agent depth
- Add "SAFETY INSPECTIONS & RECORDABLES" title above combined safety table
- Spell out "YEAR OVER YEAR COMPARISON" instead of "YoY"
- Change audit labels from "Prior Qtr" to "Prior Year" (year-over-year comparison)
- Corrective action areas template now has per-location columns for multi-campus pie charts
- Agent prompt: stronger exec summary depth requirements, C.3 multi-location emphasis
- Regenerated intake template with all layout changes

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/qbu-intake-template-v2.xlsx
+++ b/public/qbu-intake-template-v2.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="135">
   <si>
     <t>COVER SLIDE</t>
   </si>
@@ -195,16 +195,16 @@
     <t>Total</t>
   </si>
   <si>
-    <t>Prior Qtr Audits</t>
-  </si>
-  <si>
-    <t>Prior Qtr Actions</t>
-  </si>
-  <si>
-    <t>Current Qtr Audits</t>
-  </si>
-  <si>
-    <t>Current Qtr Actions</t>
+    <t>Prior Year Audits</t>
+  </si>
+  <si>
+    <t>Prior Year Actions</t>
+  </si>
+  <si>
+    <t>Current Year Audits</t>
+  </si>
+  <si>
+    <t>Current Year Actions</t>
   </si>
   <si>
     <t>Audit Change Explanation</t>
@@ -216,13 +216,10 @@
     <t>TOP CORRECTIVE ACTION AREAS</t>
   </si>
   <si>
-    <t>List the top areas where corrective actions were needed.</t>
+    <t>Use the same location names as above. Enter count of corrective actions per area per location.</t>
   </si>
   <si>
     <t>Area</t>
-  </si>
-  <si>
-    <t>Count</t>
   </si>
   <si>
     <t>Restrooms</t>
@@ -1998,13 +1995,13 @@
         <v>66</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>32</v>
@@ -2012,7 +2009,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B16" s="13" t="s">
         <v>32</v>
@@ -2029,7 +2026,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B17" s="13" t="s">
         <v>32</v>
@@ -2046,7 +2043,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>32</v>
@@ -2063,7 +2060,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B19" s="13" t="s">
         <v>32</v>
@@ -2080,7 +2077,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>32</v>
@@ -2097,7 +2094,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B21" s="13" t="s">
         <v>32</v>
@@ -2129,43 +2126,43 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B2" s="8"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B3" s="16"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B4" s="16"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" s="16"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B6" s="16"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B7" s="16"/>
     </row>
@@ -2175,31 +2172,31 @@
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B9" s="11"/>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B10" s="8"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B11" s="16"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B12" s="16"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B13" s="16"/>
     </row>
@@ -2209,43 +2206,43 @@
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" s="10"/>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B16" s="8"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B17" s="16"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B18" s="16"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B19" s="16"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B20" s="16"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B21" s="16"/>
     </row>
@@ -2267,7 +2264,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2275,7 +2272,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2289,10 +2286,10 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>87</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>88</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>32</v>
@@ -2303,7 +2300,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>32</v>
@@ -2317,7 +2314,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B6" s="13" t="s">
         <v>32</v>
@@ -2331,7 +2328,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>32</v>
@@ -2345,7 +2342,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>32</v>
@@ -2359,7 +2356,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>32</v>
@@ -2373,7 +2370,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>32</v>
@@ -2435,7 +2432,7 @@
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -2443,7 +2440,7 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -2451,10 +2448,10 @@
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>18</v>
@@ -2513,7 +2510,7 @@
     </row>
     <row r="26" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -2521,7 +2518,7 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -2532,13 +2529,13 @@
         <v>18</v>
       </c>
       <c r="B28" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="D28" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -2582,14 +2579,14 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2604,10 +2601,10 @@
         <v>18</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>102</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2647,27 +2644,27 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -2707,7 +2704,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1" s="1"/>
     </row>
@@ -2717,13 +2714,13 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B3" s="4"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B4" s="4"/>
     </row>
@@ -2733,21 +2730,21 @@
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B6" s="1"/>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>113</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>32</v>
@@ -2755,7 +2752,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B9" s="13" t="s">
         <v>32</v>
@@ -2763,7 +2760,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>32</v>
@@ -2771,7 +2768,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>32</v>
@@ -2783,37 +2780,37 @@
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B13" s="1"/>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B14" s="8"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B15" s="16"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B16" s="16"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B17" s="16"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B18" s="16"/>
     </row>
@@ -2833,14 +2830,14 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2852,13 +2849,13 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>124</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2898,32 +2895,32 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>32</v>
@@ -2934,7 +2931,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B16" s="13" t="s">
         <v>32</v>
@@ -2945,7 +2942,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B17" s="13" t="s">
         <v>32</v>
@@ -2966,14 +2963,14 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>

</xml_diff>

<commit_message>
Rebuild QBU intake template with v3 structural changes
Multi-job rows, quarterly audit tables, challenge status/quarter cols,
project location/benefit cols, editable roadmap timeline field.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/qbu-intake-template-v2.xlsx
+++ b/public/qbu-intake-template-v2.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="139">
   <si>
     <t>COVER SLIDE</t>
   </si>
@@ -45,6 +45,15 @@
     <t>Job Number</t>
   </si>
   <si>
+    <t>Job 2 Name</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Job 2 Number</t>
+  </si>
+  <si>
     <t>Region VP</t>
   </si>
   <si>
@@ -123,9 +132,6 @@
     <t>Who Notified</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>RECORDABLE INCIDENT DETAILS</t>
   </si>
   <si>
@@ -180,13 +186,7 @@
     <t>List events supported this quarter with dates.</t>
   </si>
   <si>
-    <t>OPERATIONAL AUDITS &amp; CORRECTIVE ACTIONS — Period Over Period</t>
-  </si>
-  <si>
-    <t>Enter audit and corrective action counts by location. Use actual location names.</t>
-  </si>
-  <si>
-    <t>Metric</t>
+    <t>AUDIT COUNTS BY QUARTER</t>
   </si>
   <si>
     <t>Location 1</t>
@@ -198,19 +198,22 @@
     <t>Location 3</t>
   </si>
   <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Prior Year Audits</t>
-  </si>
-  <si>
-    <t>Prior Year Actions</t>
-  </si>
-  <si>
-    <t>Current Year Audits</t>
-  </si>
-  <si>
-    <t>Current Year Actions</t>
+    <t>Location 4</t>
+  </si>
+  <si>
+    <t>CORRECTIVE ACTION COUNTS BY QUARTER</t>
+  </si>
+  <si>
+    <t>PRIOR YEAR COMPARISON</t>
+  </si>
+  <si>
+    <t>Prior Audits</t>
+  </si>
+  <si>
+    <t>Prior Actions</t>
+  </si>
+  <si>
+    <t>CHANGE EXPLANATIONS</t>
   </si>
   <si>
     <t>Audit Change Explanation</t>
@@ -219,12 +222,18 @@
     <t>Action Change Explanation</t>
   </si>
   <si>
+    <t>PER-LOCATION EXPLANATIONS</t>
+  </si>
+  <si>
+    <t>Audit Explanation</t>
+  </si>
+  <si>
+    <t>Action Explanation</t>
+  </si>
+  <si>
     <t>TOP CORRECTIVE ACTION AREAS</t>
   </si>
   <si>
-    <t>Use the same location names as above. Enter count of corrective actions per area per location.</t>
-  </si>
-  <si>
     <t>Area</t>
   </si>
   <si>
@@ -291,6 +300,9 @@
     <t>Project Description</t>
   </si>
   <si>
+    <t>Operational Benefit</t>
+  </si>
+  <si>
     <t>Renovation/Deep Clean</t>
   </si>
   <si>
@@ -336,6 +348,12 @@
     <t>Action Taken / Planned</t>
   </si>
   <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Quarter</t>
+  </si>
+  <si>
     <t>PRIOR PERIOD ACTION FOLLOW-UP</t>
   </si>
   <si>
@@ -399,40 +417,19 @@
     <t>Description &amp; Results</t>
   </si>
   <si>
-    <t>Operational Benefit</t>
-  </si>
-  <si>
     <t>UPCOMING ROADMAP</t>
   </si>
   <si>
     <t>Concrete operational items — not vague goals. Items in chronological order.</t>
   </si>
   <si>
-    <t>Month</t>
+    <t>Location / Timeline</t>
   </si>
   <si>
     <t>Initiative</t>
   </si>
   <si>
     <t>Details</t>
-  </si>
-  <si>
-    <t>Month 1</t>
-  </si>
-  <si>
-    <t>Month 2</t>
-  </si>
-  <si>
-    <t>Month 3</t>
-  </si>
-  <si>
-    <t>Month 4</t>
-  </si>
-  <si>
-    <t>Month 5</t>
-  </si>
-  <si>
-    <t>Month 6</t>
   </si>
   <si>
     <t>Period Goal Statement</t>
@@ -947,7 +944,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="36" customWidth="1"/>
@@ -1005,33 +1002,41 @@
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="4"/>
-    </row>
-    <row r="10" ht="8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-    </row>
-    <row r="11" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="1"/>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="B9" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B10" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
+      <c r="B11" s="4"/>
+    </row>
+    <row r="12" ht="8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+    </row>
+    <row r="13" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1"/>
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
@@ -1057,27 +1062,27 @@
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
     </row>
-    <row r="21" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B21" s="1"/>
-    </row>
-    <row r="22" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+    </row>
+    <row r="23" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="1"/>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
@@ -1098,6 +1103,14 @@
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="7"/>
+      <c r="B30" s="7"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="7"/>
+      <c r="B31" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1116,7 +1129,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1126,7 +1139,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1144,7 +1157,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -1154,7 +1167,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -1164,7 +1177,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -1174,7 +1187,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1192,7 +1205,7 @@
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -1202,22 +1215,22 @@
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1254,7 +1267,7 @@
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1264,22 +1277,22 @@
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1308,7 +1321,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
@@ -1326,7 +1339,7 @@
     </row>
     <row r="22" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -1336,22 +1349,22 @@
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1388,7 +1401,7 @@
     </row>
     <row r="28" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -1398,7 +1411,7 @@
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -1408,22 +1421,22 @@
     </row>
     <row r="30" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -1468,7 +1481,7 @@
     </row>
     <row r="36" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
@@ -1478,7 +1491,7 @@
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -1488,22 +1501,22 @@
     </row>
     <row r="38" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1547,7 +1560,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1557,7 +1570,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -1575,22 +1588,22 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1627,7 +1640,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -1645,7 +1658,7 @@
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1655,7 +1668,7 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -1665,22 +1678,22 @@
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1717,7 +1730,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -1735,7 +1748,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -1745,7 +1758,7 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -1771,7 +1784,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
@@ -1781,7 +1794,7 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -1845,296 +1858,471 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="36" customWidth="1"/>
-    <col min="2" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-    </row>
-    <row r="3" ht="8" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B4" s="6" t="s">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="B4" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="B5" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="B6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+      <c r="B7" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B7" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+      <c r="C19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B8" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" ht="8" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-    </row>
-    <row r="12" ht="8" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="B26" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
+      <c r="B27" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="C31" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="B32" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="B33" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="E15" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
+      <c r="B34" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B17" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B18" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
+      <c r="B39" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="B19" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
+      <c r="B40" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B20" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="B41" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D41" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>34</v>
+      <c r="B42" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B43" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B44" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C45" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
@@ -2149,43 +2337,43 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B2" s="8"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B3" s="16"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B4" s="16"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B5" s="16"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B6" s="16"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B7" s="16"/>
     </row>
@@ -2195,31 +2383,31 @@
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B9" s="11"/>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B10" s="8"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B11" s="16"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B12" s="16"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B13" s="16"/>
     </row>
@@ -2229,43 +2417,43 @@
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B15" s="10"/>
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B16" s="8"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B17" s="16"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B18" s="16"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B19" s="16"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B20" s="16"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B21" s="16"/>
     </row>
@@ -2280,14 +2468,15 @@
   <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2295,7 +2484,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2309,142 +2498,142 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>89</v>
+        <v>23</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>91</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>34</v>
+        <v>92</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>90</v>
+        <v>9</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>34</v>
+        <v>94</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>90</v>
+        <v>9</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>34</v>
+        <v>94</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>90</v>
+        <v>9</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>34</v>
+        <v>94</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>91</v>
+        <v>9</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>34</v>
+        <v>95</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>91</v>
+        <v>9</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>34</v>
+        <v>95</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>91</v>
+        <v>9</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>34</v>
+        <v>95</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" ht="8" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2455,7 +2644,7 @@
     </row>
     <row r="15" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -2463,7 +2652,7 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -2471,16 +2660,16 @@
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -2533,7 +2722,7 @@
     </row>
     <row r="26" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -2541,7 +2730,7 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -2549,16 +2738,16 @@
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -2593,23 +2782,25 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2619,96 +2810,159 @@
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="7"/>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
+      <c r="D11" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
     </row>
-    <row r="14" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>108</v>
+        <v>23</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>113</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
+        <v>114</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
+      <c r="D15" s="7"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
+      <c r="D16" s="7"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
+      <c r="D17" s="7"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>9</v>
+      </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2727,7 +2981,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B1" s="1"/>
     </row>
@@ -2737,13 +2991,13 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B3" s="4"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B4" s="4"/>
     </row>
@@ -2753,48 +3007,48 @@
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B6" s="1"/>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" ht="8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -2803,37 +3057,37 @@
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B13" s="1"/>
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B14" s="8"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B15" s="16"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B16" s="16"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B17" s="16"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B18" s="16"/>
     </row>
@@ -2853,14 +3107,14 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
@@ -2872,13 +3126,13 @@
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>126</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2918,93 +3172,93 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>132</v>
+        <v>9</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>133</v>
+        <v>9</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>134</v>
+        <v>9</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>135</v>
+        <v>9</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>136</v>
+        <v>9</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>137</v>
+        <v>9</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -3019,14 +3273,14 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>

</xml_diff>